<commit_message>
data: update 이용신청.xlsx for 2026-09-10
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/이용신청.xlsx
+++ b/docs/dashboard/data/이용신청.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="13.0" customWidth="true"/>
@@ -162,7 +162,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -172,27 +172,27 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>굴드펌프주식회사</t>
+          <t>대화항공산업(주)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2118642792</t>
+          <t>6128124764</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>이동준</t>
+          <t>강철</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>dongjun.lee@itt.com</t>
+          <t>daico.qe@daicoaero.com</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>010-2881-7914</t>
+          <t>010-7382-0072</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -209,7 +209,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -219,44 +219,44 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>하이에어코리아(주)</t>
+          <t>굴드펌프주식회사</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>6038110081</t>
+          <t>2118642792</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>황동환</t>
+          <t>이동준</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>dhhwang@hiairkorea.co.kr</t>
+          <t>dongjun.lee@itt.com</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>010-4556-5585</t>
+          <t>010-2881-7914</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-005</t>
+          <t>CN-M-26-005</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -266,44 +266,44 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>보그워너충주 유한책임회사</t>
+          <t>하이에어코리아(주)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>3038108176</t>
+          <t>6038110081</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>김혜진</t>
+          <t>황동환</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>hyejikim@borgwarner.com</t>
+          <t>dhhwang@hiairkorea.co.kr</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>010-8668-5752</t>
+          <t>010-4556-5585</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>CB-A-26-002</t>
+          <t>GN-M-26-005</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -313,37 +313,37 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>오씨아이파워 주식회사</t>
+          <t>보그워너충주 유한책임회사</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>1048644532</t>
+          <t>3038108176</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>추혜빈</t>
+          <t>김혜진</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>hyebin.chu@ocipower.co.kr</t>
+          <t>hyejikim@borgwarner.com</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>010-9193-6015</t>
+          <t>010-8668-5752</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>JB-M-26-001</t>
+          <t>CB-A-26-002</t>
         </is>
       </c>
     </row>
@@ -360,37 +360,37 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
+          <t>오씨아이파워 주식회사</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>7888101296</t>
+          <t>1048644532</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>박은범</t>
+          <t>추혜빈</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Owen_Park@sgssemi.com</t>
+          <t>hyebin.chu@ocipower.co.kr</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>010-9335-4934</t>
+          <t>010-9193-6015</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-004</t>
+          <t>JB-M-26-001</t>
         </is>
       </c>
     </row>
@@ -407,27 +407,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
+          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>8858800321</t>
+          <t>7888101296</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>사금석</t>
+          <t>박은범</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>gssa@vtekorea.com</t>
+          <t>Owen_Park@sgssemi.com</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>010-8832-0250</t>
+          <t>010-9335-4934</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -437,7 +437,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-005</t>
+          <t>GG-E-26-004</t>
         </is>
       </c>
     </row>
@@ -454,27 +454,27 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에이치엔에프</t>
+          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>7398801954</t>
+          <t>8858800321</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>조수형</t>
+          <t>사금석</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>whtngud17@hnfvac.com</t>
+          <t>gssa@vtekorea.com</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>010-2310-3404</t>
+          <t>010-8832-0250</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -484,7 +484,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-002</t>
+          <t>GG-E-26-005</t>
         </is>
       </c>
     </row>
@@ -501,37 +501,37 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>디지트론</t>
+          <t>주식회사 에이치엔에프</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>1298603001</t>
+          <t>7398801954</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>정재종</t>
+          <t>조수형</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>jjjeong@digitron.kr</t>
+          <t>whtngud17@hnfvac.com</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>010-4511-4977</t>
+          <t>010-2310-3404</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-012</t>
+          <t>CN-M-26-002</t>
         </is>
       </c>
     </row>
@@ -548,37 +548,37 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>(주)센추리 아산공장</t>
+          <t>디지트론</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>3128545076</t>
+          <t>1298603001</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>허민영</t>
+          <t>정재종</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>myheo3153@century.co.kr</t>
+          <t>jjjeong@digitron.kr</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>010-8484-3476</t>
+          <t>010-4511-4977</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-003</t>
+          <t>GG-M-26-012</t>
         </is>
       </c>
     </row>
@@ -595,27 +595,27 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>세일전장 주식회사</t>
+          <t>(주)센추리 아산공장</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2218802452</t>
+          <t>3128545076</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>홍유성</t>
+          <t>허민영</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>seic97@ehe.kr</t>
+          <t>myheo3153@century.co.kr</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>010-4054-0831</t>
+          <t>010-8484-3476</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>CN-A-26-002</t>
+          <t>CN-M-26-003</t>
         </is>
       </c>
     </row>
@@ -642,27 +642,27 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>(주)동광보일러</t>
+          <t>세일전장 주식회사</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>1408121883</t>
+          <t>2218802452</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>김용휘</t>
+          <t>홍유성</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>dydgnl153@krb.co.kr</t>
+          <t>seic97@ehe.kr</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>010-9731-5222</t>
+          <t>010-4054-0831</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-004</t>
+          <t>CN-A-26-002</t>
         </is>
       </c>
     </row>
@@ -689,27 +689,27 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>(주)윤성에프앤씨</t>
+          <t>(주)동광보일러</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>1348150350</t>
+          <t>1408121883</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>윤성현</t>
+          <t>김용휘</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>shyun@ysfc.co.kr</t>
+          <t>dydgnl153@krb.co.kr</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>010-9914-7989</t>
+          <t>010-9731-5222</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -719,54 +719,54 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-005</t>
+          <t>CN-M-26-004</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>한국에스엠씨 주식회사</t>
+          <t>(주)윤성에프앤씨</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1368505145</t>
+          <t>1348150350</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>신창재</t>
+          <t>윤성현</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>mom14@nate.com</t>
+          <t>shyun@ysfc.co.kr</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>010-6293-5314</t>
+          <t>010-9914-7989</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>GG-M-26-005</t>
         </is>
       </c>
     </row>
@@ -783,12 +783,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>한국요꼬가와일렉트로닉스매뉴팩처링(주)</t>
+          <t>한국에스엠씨 주식회사</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>1228171556</t>
+          <t>1368505145</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -867,37 +867,37 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>대기</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>한국의료기기평가원</t>
+          <t>한국요꼬가와일렉트로닉스매뉴팩처링(주)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>1298210386</t>
+          <t>1228171556</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>김준수</t>
+          <t>신창재</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>kjunsjs@kimda.or.kr</t>
+          <t>mom14@nate.com</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>010-7257-0023</t>
+          <t>010-6293-5314</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -914,47 +914,47 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>대기</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>비카코리아 주식회사</t>
+          <t>한국의료기기평가원</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>6108128707</t>
+          <t>1298210386</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>이진형</t>
+          <t>김준수</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>jinhyoung.Lee@wika.com</t>
+          <t>kjunsjs@kimda.or.kr</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>010-4026-3019</t>
+          <t>010-7257-0023</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t/>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-002</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -971,27 +971,27 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>(주)디바이스</t>
+          <t>비카코리아 주식회사</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>3128157991</t>
+          <t>6108128707</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>김용호</t>
+          <t>이진형</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>kimyh@deviceeng.co.kr</t>
+          <t>jinhyoung.Lee@wika.com</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>010-3474-3716</t>
+          <t>010-4026-3019</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1001,14 +1001,14 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>CN-E-26-001</t>
+          <t>GG-M-26-002</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1018,37 +1018,37 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>(주)케이피씨엠</t>
+          <t>(주)디바이스</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>5158140973</t>
+          <t>3128157991</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>이예슬</t>
+          <t>김용호</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>ys-lee@kpccorp.co.kr</t>
+          <t>kimyh@deviceeng.co.kr</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>010-9721-4885</t>
+          <t>010-3474-3716</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>GB-M-26-001</t>
+          <t>CN-E-26-001</t>
         </is>
       </c>
     </row>
@@ -1065,27 +1065,27 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>지에프에스</t>
+          <t>(주)케이피씨엠</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>1278107419</t>
+          <t>5158140973</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>임승현</t>
+          <t>이예슬</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>skyies88@gfs.co.kr</t>
+          <t>ys-lee@kpccorp.co.kr</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>010-9516-5508</t>
+          <t>010-9721-4885</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-003</t>
+          <t>GB-M-26-001</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1137,59 +1137,59 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>GG-E-26-003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>에브제트아시아</t>
+          <t>지에프에스</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>1208731282</t>
+          <t>1278107419</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>전승헌</t>
+          <t>임승현</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>sh.chun@avjet.kr</t>
+          <t>skyies88@gfs.co.kr</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>010-8833-0349</t>
+          <t>010-9516-5508</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t/>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>SE-S-26-001</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1206,27 +1206,27 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>코리아하이텍</t>
+          <t>에브제트아시아</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1348106311</t>
+          <t>1208731282</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>박진우</t>
+          <t>전승헌</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>jwp97@koreahitek.co.kr</t>
+          <t>sh.chun@avjet.kr</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>010-6377-6757</t>
+          <t>010-8833-0349</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-002</t>
+          <t>SE-S-26-001</t>
         </is>
       </c>
     </row>
@@ -1253,27 +1253,27 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>(주)경인기술</t>
+          <t>코리아하이텍</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>1138156416</t>
+          <t>1348106311</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>임성종</t>
+          <t>박진우</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>tjdwhd8809@naver.com</t>
+          <t>jwp97@koreahitek.co.kr</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>010-2905-7307</t>
+          <t>010-6377-6757</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>SE-E-26-002</t>
+          <t>GG-E-26-002</t>
         </is>
       </c>
     </row>
@@ -1295,42 +1295,42 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>대기</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>에스에이치테크</t>
+          <t>(주)경인기술</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>8818100276</t>
+          <t>1138156416</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>정가브리엘</t>
+          <t>임성종</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>jgadco28@shtech9080.com</t>
+          <t>tjdwhd8809@naver.com</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>010-8789-9924</t>
+          <t>010-2905-7307</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>SE-E-26-002</t>
         </is>
       </c>
     </row>
@@ -1342,42 +1342,42 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>대기</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>(주)알피바이오</t>
+          <t>에스에이치테크</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>7758501361</t>
+          <t>8818100276</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>노승우</t>
+          <t>정가브리엘</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>nswok03@rpcorp.co.kr</t>
+          <t>jgadco28@shtech9080.com</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>010-4899-3983</t>
+          <t>010-8789-9924</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t/>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>GG-B-26-001</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1394,27 +1394,27 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>씨트론(주)</t>
+          <t>(주)알피바이오</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1228159023</t>
+          <t>7758501361</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>양혜원</t>
+          <t>노승우</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>hyewon.yang@seetron.co.kr</t>
+          <t>nswok03@rpcorp.co.kr</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>010-2770-7226</t>
+          <t>010-4899-3983</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-001</t>
+          <t>GG-B-26-001</t>
         </is>
       </c>
     </row>
@@ -1441,27 +1441,27 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>코젠바이오텍</t>
+          <t>씨트론(주)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>1018156320</t>
+          <t>1228159023</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>정지만</t>
+          <t>양혜원</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>stopman@kogene.co.kr</t>
+          <t>hyewon.yang@seetron.co.kr</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>010-5348-2308</t>
+          <t>010-2770-7226</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>SE-B-26-001</t>
+          <t>GG-M-26-001</t>
         </is>
       </c>
     </row>
@@ -1488,27 +1488,27 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>주식회사 덱스레보</t>
+          <t>코젠바이오텍</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1198678150</t>
+          <t>1018156320</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>이득훈</t>
+          <t>정지만</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>dh.lee@dexlevo.com</t>
+          <t>stopman@kogene.co.kr</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>010-4119-7124</t>
+          <t>010-5348-2308</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1518,14 +1518,14 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>SE-M-26-006</t>
+          <t>SE-B-26-001</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1535,27 +1535,27 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>디엔엠항공</t>
+          <t>주식회사 덱스레보</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>6131783159</t>
+          <t>1198678150</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>김미희</t>
+          <t>이득훈</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>dnma@dnmaero.com</t>
+          <t>dh.lee@dexlevo.com</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>010-8131-0888</t>
+          <t>010-4119-7124</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-003</t>
+          <t>SE-M-26-006</t>
         </is>
       </c>
     </row>
@@ -1582,37 +1582,37 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>대성티엠씨</t>
+          <t>디엔엠항공</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>6068641818</t>
+          <t>6131783159</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>유신재</t>
+          <t>김미희</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>daesungaero@hanmail.net</t>
+          <t>dnma@dnmaero.com</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>010-5307-6284</t>
+          <t>010-8131-0888</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-004</t>
+          <t>GN-M-26-003</t>
         </is>
       </c>
     </row>
@@ -1624,42 +1624,42 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>카프마이크로</t>
+          <t>대성티엠씨</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>3148613655</t>
+          <t>6068641818</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>김호영</t>
+          <t>유신재</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>hoykim@caphmicro.com</t>
+          <t>daesungaero@hanmail.net</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>010-3224-7480</t>
+          <t>010-5307-6284</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>GN-M-26-004</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1686,27 +1686,27 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>박준영</t>
+          <t>김호영</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>jypark@caphmicro.com</t>
+          <t>hoykim@caphmicro.com</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>010-9305-1034</t>
+          <t>010-3224-7480</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t/>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-002</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1718,42 +1718,42 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>(주)한국인삼공사</t>
+          <t>카프마이크로</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>3148123992</t>
+          <t>3148613655</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>이건영</t>
+          <t>박준영</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>20200074@kgc.co.kr</t>
+          <t>jypark@caphmicro.com</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>010-7126-4089</t>
+          <t>010-9305-1034</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>GN-M-26-002</t>
         </is>
       </c>
     </row>
@@ -1765,89 +1765,89 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>연합정밀(주)</t>
+          <t>(주)한국인삼공사</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>3128109219</t>
+          <t>3148123992</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>하상우</t>
+          <t>이건영</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>swha@yeonhab.co.kr</t>
+          <t>20200074@kgc.co.kr</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>010-2942-3411</t>
+          <t>010-7126-4089</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-001</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>주식회사 신화프리텍</t>
+          <t>연합정밀(주)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>6088151660</t>
+          <t>3128109219</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>김혜민</t>
+          <t>하상우</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>hmkim@shinhwa-pritech.com</t>
+          <t>swha@yeonhab.co.kr</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>010-2540-7649</t>
+          <t>010-2942-3411</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>CN-M-26-001</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>(주)신화프리텍</t>
+          <t>주식회사 신화프리텍</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1874,27 +1874,27 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>최문정</t>
+          <t>김혜민</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>mjchoi@shinhwa-pritech.com</t>
+          <t>hmkim@shinhwa-pritech.com</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>010-8669-1533</t>
+          <t>010-2540-7649</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t/>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-001</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1911,27 +1911,27 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>(주)한국기능공사</t>
+          <t>(주)신화프리텍</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>1258112293</t>
+          <t>6088151660</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>하갑봉</t>
+          <t>최문정</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>gbha@hkcb.co.kr</t>
+          <t>mjchoi@shinhwa-pritech.com</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>010-5655-3719</t>
+          <t>010-8669-1533</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -1941,14 +1941,14 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>CB-A-26-001</t>
+          <t>GN-M-26-001</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1958,37 +1958,37 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>주식회사 웨이투웨이</t>
+          <t>(주)한국기능공사</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>1408181673</t>
+          <t>1258112293</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>김미선</t>
+          <t>하갑봉</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>ms4564@wtwkorea.co.kr</t>
+          <t>gbha@hkcb.co.kr</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>010-9301-4564</t>
+          <t>010-5655-3719</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-002</t>
+          <t>CB-A-26-001</t>
         </is>
       </c>
     </row>
@@ -2005,35 +2005,82 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
+          <t>주식회사 웨이투웨이</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>1408181673</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>김미선</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>ms4564@wtwkorea.co.kr</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>010-9301-4564</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>GG-S-26-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>승인</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
           <t>(주)서연이화 아산공장</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>3128564374</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>류제형</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>jh.ryoo@seoyoneh.com</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>010-8210-1082</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>CN-A-26-001</t>
         </is>

</xml_diff>

<commit_message>
data: update 이용신청.xlsx for 2026-09-18
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/이용신청.xlsx
+++ b/docs/dashboard/data/이용신청.xlsx
@@ -919,7 +919,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>대기</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -949,12 +949,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>GG-S-26-005</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>대기</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data: update 이용신청.xlsx for 2026-09-23
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/이용신청.xlsx
+++ b/docs/dashboard/data/이용신청.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="13.0" customWidth="true"/>
@@ -162,7 +162,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -172,27 +172,27 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>대화항공산업(주)</t>
+          <t>이코리아산업</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>6128124764</t>
+          <t>6218141146</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>강철</t>
+          <t>최준호</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>daico.qe@daicoaero.com</t>
+          <t>q@ecoreaind.com</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>010-7382-0072</t>
+          <t>010-2592-0114</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -209,148 +209,148 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>대기</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>굴드펌프주식회사</t>
+          <t>삼동허브 (주)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2118642792</t>
+          <t>6218123584</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>이동준</t>
+          <t>이성욱</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>dongjun.lee@itt.com</t>
+          <t>leesuwo@samdonghub.com</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>010-2881-7914</t>
+          <t>010-3218-0014</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t/>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-005</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>하이에어코리아(주)</t>
+          <t>(주)신우테크</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>6038110081</t>
+          <t>1258137969</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>황동환</t>
+          <t>박재희</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>dhhwang@hiairkorea.co.kr</t>
+          <t>pbc044@naver.com</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>010-4556-5585</t>
+          <t>010-5258-3374</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t/>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-005</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>대기</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>보그워너충주 유한책임회사</t>
+          <t>대화항공산업(주)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>3038108176</t>
+          <t>6128124764</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>김혜진</t>
+          <t>강철</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>hyejikim@borgwarner.com</t>
+          <t>daico.qe@daicoaero.com</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>010-8668-5752</t>
+          <t>010-7382-0072</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t/>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>CB-A-26-002</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -360,44 +360,44 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>오씨아이파워 주식회사</t>
+          <t>굴드펌프주식회사</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>1048644532</t>
+          <t>2118642792</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>추혜빈</t>
+          <t>이동준</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>hyebin.chu@ocipower.co.kr</t>
+          <t>dongjun.lee@itt.com</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>010-9193-6015</t>
+          <t>010-2881-7914</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>JB-M-26-001</t>
+          <t>CN-M-26-005</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -407,44 +407,44 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
+          <t>하이에어코리아(주)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>7888101296</t>
+          <t>6038110081</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>박은범</t>
+          <t>황동환</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Owen_Park@sgssemi.com</t>
+          <t>dhhwang@hiairkorea.co.kr</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>010-9335-4934</t>
+          <t>010-4556-5585</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-004</t>
+          <t>GN-M-26-005</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -454,37 +454,37 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
+          <t>보그워너충주 유한책임회사</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>8858800321</t>
+          <t>3038108176</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>사금석</t>
+          <t>김혜진</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>gssa@vtekorea.com</t>
+          <t>hyejikim@borgwarner.com</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>010-8832-0250</t>
+          <t>010-8668-5752</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-005</t>
+          <t>CB-A-26-002</t>
         </is>
       </c>
     </row>
@@ -501,37 +501,37 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에이치엔에프</t>
+          <t>오씨아이파워 주식회사</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>7398801954</t>
+          <t>1048644532</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>조수형</t>
+          <t>추혜빈</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>whtngud17@hnfvac.com</t>
+          <t>hyebin.chu@ocipower.co.kr</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>010-2310-3404</t>
+          <t>010-9193-6015</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-002</t>
+          <t>JB-M-26-001</t>
         </is>
       </c>
     </row>
@@ -548,37 +548,37 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>디지트론</t>
+          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>1298603001</t>
+          <t>7888101296</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>정재종</t>
+          <t>박은범</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>jjjeong@digitron.kr</t>
+          <t>Owen_Park@sgssemi.com</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>010-4511-4977</t>
+          <t>010-9335-4934</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-012</t>
+          <t>GG-E-26-004</t>
         </is>
       </c>
     </row>
@@ -595,27 +595,27 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>(주)센추리 아산공장</t>
+          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>3128545076</t>
+          <t>8858800321</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>허민영</t>
+          <t>사금석</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>myheo3153@century.co.kr</t>
+          <t>gssa@vtekorea.com</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>010-8484-3476</t>
+          <t>010-8832-0250</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-003</t>
+          <t>GG-E-26-005</t>
         </is>
       </c>
     </row>
@@ -642,27 +642,27 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>세일전장 주식회사</t>
+          <t>주식회사 에이치엔에프</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2218802452</t>
+          <t>7398801954</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>홍유성</t>
+          <t>조수형</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>seic97@ehe.kr</t>
+          <t>whtngud17@hnfvac.com</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>010-4054-0831</t>
+          <t>010-2310-3404</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>CN-A-26-002</t>
+          <t>CN-M-26-002</t>
         </is>
       </c>
     </row>
@@ -689,37 +689,37 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>(주)동광보일러</t>
+          <t>디지트론</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>1408121883</t>
+          <t>1298603001</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>김용휘</t>
+          <t>정재종</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>dydgnl153@krb.co.kr</t>
+          <t>jjjeong@digitron.kr</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>010-9731-5222</t>
+          <t>010-4511-4977</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-004</t>
+          <t>GG-M-26-012</t>
         </is>
       </c>
     </row>
@@ -736,27 +736,27 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>(주)윤성에프앤씨</t>
+          <t>(주)센추리 아산공장</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1348150350</t>
+          <t>3128545076</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>윤성현</t>
+          <t>허민영</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>shyun@ysfc.co.kr</t>
+          <t>myheo3153@century.co.kr</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>010-9914-7989</t>
+          <t>010-8484-3476</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -766,296 +766,296 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-005</t>
+          <t>CN-M-26-003</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>한국에스엠씨 주식회사</t>
+          <t>세일전장 주식회사</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>1368505145</t>
+          <t>2218802452</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>신창재</t>
+          <t>홍유성</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>mom14@nate.com</t>
+          <t>seic97@ehe.kr</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>010-6293-5314</t>
+          <t>010-4054-0831</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>CN-A-26-002</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>한국요꼬가와일렉트로닉스매뉴팩처링(주)</t>
+          <t>(주)동광보일러</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>1228171556</t>
+          <t>1408121883</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>신창재</t>
+          <t>김용휘</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>mom14@nate.com</t>
+          <t>dydgnl153@krb.co.kr</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>010-6293-5314</t>
+          <t>010-9731-5222</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>CN-M-26-004</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>한국요꼬가와일렉트로닉스매뉴팩처링(주)</t>
+          <t>(주)윤성에프앤씨</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>1228171556</t>
+          <t>1348150350</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>신창재</t>
+          <t>윤성현</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>mom14@nate.com</t>
+          <t>shyun@ysfc.co.kr</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>010-6293-5314</t>
+          <t>010-9914-7989</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>GG-M-26-005</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>한국의료기기평가원</t>
+          <t>한국에스엠씨 주식회사</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>1298210386</t>
+          <t>1368505145</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>김준수</t>
+          <t>신창재</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>kjunsjs@kimda.or.kr</t>
+          <t>mom14@nate.com</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>010-7257-0023</t>
+          <t>010-6293-5314</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-005</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>비카코리아 주식회사</t>
+          <t>한국요꼬가와일렉트로닉스매뉴팩처링(주)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>6108128707</t>
+          <t>1228171556</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>이진형</t>
+          <t>신창재</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>jinhyoung.Lee@wika.com</t>
+          <t>mom14@nate.com</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>010-4026-3019</t>
+          <t>010-6293-5314</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t/>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-002</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>(주)디바이스</t>
+          <t>한국요꼬가와일렉트로닉스매뉴팩처링(주)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>3128157991</t>
+          <t>1228171556</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>김용호</t>
+          <t>신창재</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>kimyh@deviceeng.co.kr</t>
+          <t>mom14@nate.com</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>010-3474-3716</t>
+          <t>010-6293-5314</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t/>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>CN-E-26-001</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1065,44 +1065,44 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>(주)케이피씨엠</t>
+          <t>한국의료기기평가원</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>5158140973</t>
+          <t>1298210386</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>이예슬</t>
+          <t>김준수</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>ys-lee@kpccorp.co.kr</t>
+          <t>kjunsjs@kimda.or.kr</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>010-9721-4885</t>
+          <t>010-7257-0023</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>GB-M-26-001</t>
+          <t>GG-S-26-005</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1112,91 +1112,91 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>지에프에스</t>
+          <t>비카코리아 주식회사</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>1278107419</t>
+          <t>6108128707</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>임승현</t>
+          <t>이진형</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>skyies88@gfs.co.kr</t>
+          <t>jinhyoung.Lee@wika.com</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>010-9516-5508</t>
+          <t>010-4026-3019</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-003</t>
+          <t>GG-M-26-002</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>지에프에스</t>
+          <t>(주)디바이스</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>1278107419</t>
+          <t>3128157991</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>임승현</t>
+          <t>김용호</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>skyies88@gfs.co.kr</t>
+          <t>kimyh@deviceeng.co.kr</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>010-9516-5508</t>
+          <t>010-3474-3716</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>CN-E-26-001</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1206,44 +1206,44 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>에브제트아시아</t>
+          <t>(주)케이피씨엠</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1208731282</t>
+          <t>5158140973</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>전승헌</t>
+          <t>이예슬</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>sh.chun@avjet.kr</t>
+          <t>ys-lee@kpccorp.co.kr</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>010-8833-0349</t>
+          <t>010-9721-4885</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>SE-S-26-001</t>
+          <t>GB-M-26-001</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1253,84 +1253,84 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>코리아하이텍</t>
+          <t>지에프에스</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>1348106311</t>
+          <t>1278107419</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>박진우</t>
+          <t>임승현</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>jwp97@koreahitek.co.kr</t>
+          <t>skyies88@gfs.co.kr</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>010-6377-6757</t>
+          <t>010-9516-5508</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-002</t>
+          <t>GG-E-26-003</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>(주)경인기술</t>
+          <t>지에프에스</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>1138156416</t>
+          <t>1278107419</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>임성종</t>
+          <t>임승현</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>tjdwhd8809@naver.com</t>
+          <t>skyies88@gfs.co.kr</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>010-2905-7307</t>
+          <t>010-9516-5508</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t/>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>SE-E-26-002</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1342,42 +1342,42 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>에스에이치테크</t>
+          <t>에브제트아시아</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>8818100276</t>
+          <t>1208731282</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>정가브리엘</t>
+          <t>전승헌</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>jgadco28@shtech9080.com</t>
+          <t>sh.chun@avjet.kr</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>010-8789-9924</t>
+          <t>010-8833-0349</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>SE-S-26-001</t>
         </is>
       </c>
     </row>
@@ -1394,27 +1394,27 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>(주)알피바이오</t>
+          <t>코리아하이텍</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>7758501361</t>
+          <t>1348106311</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>노승우</t>
+          <t>박진우</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>nswok03@rpcorp.co.kr</t>
+          <t>jwp97@koreahitek.co.kr</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>010-4899-3983</t>
+          <t>010-6377-6757</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>GG-B-26-001</t>
+          <t>GG-E-26-002</t>
         </is>
       </c>
     </row>
@@ -1441,27 +1441,27 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>씨트론(주)</t>
+          <t>(주)경인기술</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>1228159023</t>
+          <t>1138156416</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>양혜원</t>
+          <t>임성종</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>hyewon.yang@seetron.co.kr</t>
+          <t>tjdwhd8809@naver.com</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>010-2770-7226</t>
+          <t>010-2905-7307</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-001</t>
+          <t>SE-E-26-002</t>
         </is>
       </c>
     </row>
@@ -1483,42 +1483,42 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>코젠바이오텍</t>
+          <t>에스에이치테크</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1018156320</t>
+          <t>8818100276</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>정지만</t>
+          <t>정가브리엘</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>stopman@kogene.co.kr</t>
+          <t>jgadco28@shtech9080.com</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>010-5348-2308</t>
+          <t>010-8789-9924</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t/>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>SE-B-26-001</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1535,27 +1535,27 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>주식회사 덱스레보</t>
+          <t>(주)알피바이오</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>1198678150</t>
+          <t>7758501361</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>이득훈</t>
+          <t>노승우</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>dh.lee@dexlevo.com</t>
+          <t>nswok03@rpcorp.co.kr</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>010-4119-7124</t>
+          <t>010-4899-3983</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1565,14 +1565,14 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>SE-M-26-006</t>
+          <t>GG-B-26-001</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1582,27 +1582,27 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>디엔엠항공</t>
+          <t>씨트론(주)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>6131783159</t>
+          <t>1228159023</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>김미희</t>
+          <t>양혜원</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>dnma@dnmaero.com</t>
+          <t>hyewon.yang@seetron.co.kr</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>010-8131-0888</t>
+          <t>010-2770-7226</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1612,14 +1612,14 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-003</t>
+          <t>GG-M-26-001</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1629,84 +1629,84 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>대성티엠씨</t>
+          <t>코젠바이오텍</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>6068641818</t>
+          <t>1018156320</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>유신재</t>
+          <t>정지만</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>daesungaero@hanmail.net</t>
+          <t>stopman@kogene.co.kr</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>010-5307-6284</t>
+          <t>010-5348-2308</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-004</t>
+          <t>SE-B-26-001</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>카프마이크로</t>
+          <t>주식회사 덱스레보</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>3148613655</t>
+          <t>1198678150</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>김호영</t>
+          <t>이득훈</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>hoykim@caphmicro.com</t>
+          <t>dh.lee@dexlevo.com</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>010-3224-7480</t>
+          <t>010-4119-7124</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>SE-M-26-006</t>
         </is>
       </c>
     </row>
@@ -1723,37 +1723,37 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>카프마이크로</t>
+          <t>디엔엠항공</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>3148613655</t>
+          <t>6131783159</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>박준영</t>
+          <t>김미희</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>jypark@caphmicro.com</t>
+          <t>dnma@dnmaero.com</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>010-9305-1034</t>
+          <t>010-8131-0888</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-002</t>
+          <t>GN-M-26-003</t>
         </is>
       </c>
     </row>
@@ -1765,42 +1765,42 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>(주)한국인삼공사</t>
+          <t>대성티엠씨</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>3148123992</t>
+          <t>6068641818</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>이건영</t>
+          <t>유신재</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>20200074@kgc.co.kr</t>
+          <t>daesungaero@hanmail.net</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>010-7126-4089</t>
+          <t>010-5307-6284</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>GN-M-26-004</t>
         </is>
       </c>
     </row>
@@ -1812,143 +1812,143 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>연합정밀(주)</t>
+          <t>카프마이크로</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>3128109219</t>
+          <t>3148613655</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>하상우</t>
+          <t>김호영</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>swha@yeonhab.co.kr</t>
+          <t>hoykim@caphmicro.com</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>010-2942-3411</t>
+          <t>010-3224-7480</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t/>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-001</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>반려</t>
+          <t>승인</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>주식회사 신화프리텍</t>
+          <t>카프마이크로</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>6088151660</t>
+          <t>3148613655</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>김혜민</t>
+          <t>박준영</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>hmkim@shinhwa-pritech.com</t>
+          <t>jypark@caphmicro.com</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>010-2540-7649</t>
+          <t>010-9305-1034</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>GN-M-26-002</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>(주)신화프리텍</t>
+          <t>(주)한국인삼공사</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>6088151660</t>
+          <t>3148123992</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>최문정</t>
+          <t>이건영</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>mjchoi@shinhwa-pritech.com</t>
+          <t>20200074@kgc.co.kr</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>010-8669-1533</t>
+          <t>010-7126-4089</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-001</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1958,129 +1958,270 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>(주)한국기능공사</t>
+          <t>연합정밀(주)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>1258112293</t>
+          <t>3128109219</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>하갑봉</t>
+          <t>하상우</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>gbha@hkcb.co.kr</t>
+          <t>swha@yeonhab.co.kr</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>010-5655-3719</t>
+          <t>010-2942-3411</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>CB-A-26-001</t>
+          <t>CN-M-26-001</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>승인</t>
+          <t>반려</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>주식회사 웨이투웨이</t>
+          <t>주식회사 신화프리텍</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>1408181673</t>
+          <t>6088151660</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>김미선</t>
+          <t>김혜민</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>ms4564@wtwkorea.co.kr</t>
+          <t>hmkim@shinhwa-pritech.com</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>010-9301-4564</t>
+          <t>010-2540-7649</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t/>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-002</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>승인</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>(주)신화프리텍</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>6088151660</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>최문정</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>mjchoi@shinhwa-pritech.com</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>010-8669-1533</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>GN-M-26-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>승인</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>(주)한국기능공사</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>1258112293</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>하갑봉</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>gbha@hkcb.co.kr</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>010-5655-3719</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>CB-A-26-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>승인</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>승인</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>주식회사 웨이투웨이</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>1408181673</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>김미선</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>ms4564@wtwkorea.co.kr</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>010-9301-4564</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>GG-S-26-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>승인</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>(주)서연이화 아산공장</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>3128564374</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>류제형</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>jh.ryoo@seoyoneh.com</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>010-8210-1082</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>CN-A-26-001</t>
         </is>

</xml_diff>